<commit_message>
Egypt: RSDS reservation terms quoted (day passes, rental, deposit, cancellation), budget re-cut to USD 1,300 / 1,250, RSDS-versus-Blue Ocean comparison for George; TDI correction sent
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0169irXwrgR4zfoxWYodwM9b
</commit_message>
<xml_diff>
--- a/december-plan/pricing/egypt_group_budget.xlsx
+++ b/december-plan/pricing/egypt_group_budget.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="160">
   <si>
     <t xml:space="preserve">Egypt group budget — inputs (blue cells are editable; EUR unless stated)</t>
   </si>
@@ -91,7 +91,7 @@
     <t xml:space="preserve">EUR/night</t>
   </si>
   <si>
-    <t xml:space="preserve">QUOTED (six-night quote; five-night rate asked)</t>
+    <t xml:space="preserve">QUOTED 26 Sep (390 for five nights; Deluxe Chalet 113/night = 565)</t>
   </si>
   <si>
     <t xml:space="preserve">Nights, Sun 3 – Fri 8 Jan</t>
@@ -103,19 +103,19 @@
     <t xml:space="preserve">programme</t>
   </si>
   <si>
-    <t xml:space="preserve">House reef diving package, 5 days unlimited (certified)</t>
+    <t xml:space="preserve">House reef diving, four one-day unlimited passes Mon–Thu (certified), EUR 77 a day</t>
   </si>
   <si>
     <t xml:space="preserve">EUR</t>
   </si>
   <si>
-    <t xml:space="preserve">QUOTED; four-day package asked, keep 5-day until answered</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Extra house-reef day (used for the new divers' Thursday after certification)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QUOTED as the 6th-day add-on; ASSUMED usable as a single day</t>
+    <t xml:space="preserve">QUOTED 26 Sep (no four-day package; cheaper than the five-day 347)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One-day unlimited house-reef pass (the new divers' Thursday after certification)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 26 Sep</t>
   </si>
   <si>
     <t xml:space="preserve">Open Water course incl. equipment</t>
@@ -148,13 +148,13 @@
     <t xml:space="preserve">Environmental fee 10 + hyperbaric fee 7, once per person</t>
   </si>
   <si>
-    <t xml:space="preserve">Full equipment rental per day, certified divers (course prices include gear)</t>
+    <t xml:space="preserve">Full equipment rental incl. computer per day, certified divers (course prices include gear)</t>
   </si>
   <si>
     <t xml:space="preserve">EUR/day</t>
   </si>
   <si>
-    <t xml:space="preserve">ASSUMED; asked 24 Sep</t>
+    <t xml:space="preserve">QUOTED 26 Sep (33 without computer; club rule: computers inside the fee)</t>
   </si>
   <si>
     <t xml:space="preserve">Rental days, certified (Mon–Thu)</t>
@@ -175,7 +175,10 @@
     <t xml:space="preserve">QUOTED; modelled as 11, 21, 30</t>
   </si>
   <si>
-    <t xml:space="preserve">RSDS deposit at booking</t>
+    <t xml:space="preserve">RSDS deposit at booking (non-refundable)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">QUOTED 26 Sep; balance on site, 5% off for cash, card +3%</t>
   </si>
   <si>
     <t xml:space="preserve">Leader costs carried by the group (George's lodging and diving come from the first free place)</t>
@@ -223,10 +226,7 @@
     <t xml:space="preserve">DOCUMENTED (secondary): USD 30 since 1 Mar 2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Meet-and-assist at the airport (optional)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">QUOTE NEEDED; asked 24 Sep</t>
+    <t xml:space="preserve">Visa on arrival plus meet-and-assist at the airport (optional, minimum four)</t>
   </si>
   <si>
     <t xml:space="preserve">Drinks, snacks, tips per day (full board covers meals)</t>
@@ -253,7 +253,7 @@
     <t xml:space="preserve">Certified diver</t>
   </si>
   <si>
-    <t xml:space="preserve">Diving with RSDS (course + e-code + Thursday day, or 5-day house reef package)</t>
+    <t xml:space="preserve">Diving with RSDS (course + e-code + Thursday pass, or four day passes Mon–Thu)</t>
   </si>
   <si>
     <t xml:space="preserve">Dolphin House day boat incl. park fee (certified, Wed)</t>
@@ -283,7 +283,7 @@
     <t xml:space="preserve">Fee in USD before rounding</t>
   </si>
   <si>
-    <t xml:space="preserve">TRIP FEE, USD (rounded up to the nearest 100, as posted)</t>
+    <t xml:space="preserve">TRIP FEE, USD (rounded up to the nearest 50, as posted)</t>
   </si>
   <si>
     <t xml:space="preserve">Optional add-ons at sign-up, charged at cost (USD)</t>
@@ -406,7 +406,7 @@
     <t xml:space="preserve">George's pot, EUR: value of spare free places (no commission offered)</t>
   </si>
   <si>
-    <t xml:space="preserve">Deposits and cash (RSDS terms ASSUMED until answered)</t>
+    <t xml:space="preserve">Deposits and cash (RSDS: 20% non-refundable at booking, balance on site)</t>
   </si>
   <si>
     <t xml:space="preserve">Participant deposits at sign-up (USD 400 each, in EUR)</t>
@@ -418,10 +418,10 @@
     <t xml:space="preserve">Deposit cover (positive means deposits fund the outflow)</t>
   </si>
   <si>
-    <t xml:space="preserve">Notes: fees are posted in USD and converted at the workbook rate, so a weaker dollar eats the surplus first; the contingency and the 12-person floor are the cushion. A free place beyond George's own is credited to the club here; George can instead ask to keep it as his pot (Tec 40 course, asked 24 Sep).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Payment schedule (RSDS deposit and cancellation terms asked 24 Sep; dates provisional)</t>
+    <t xml:space="preserve">Notes: fees are posted in USD and converted at the workbook rate, so a weaker dollar eats the surplus first; the contingency and the 12-person floor are the cushion. A free place beyond George's own is credited to the club here; George can instead ask to keep it as his pot (a TDI course, parked). Paying the balance in cash on site earns a 5% discount on the RSDS invoice, not modelled.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Payment schedule (RSDS terms quoted 26 Sep; dates provisional)</t>
   </si>
   <si>
     <t xml:space="preserve">date</t>
@@ -454,7 +454,7 @@
     <t xml:space="preserve">by Fri 23 Oct</t>
   </si>
   <si>
-    <t xml:space="preserve">RSDS deposit (share to confirm); e-codes issued to students</t>
+    <t xml:space="preserve">RSDS deposit, 20% of the invoice, non-refundable, by bank transfer or card; e-codes issued to students</t>
   </si>
   <si>
     <t xml:space="preserve">club account</t>
@@ -466,10 +466,13 @@
     <t xml:space="preserve">Participant balances due (fee less deposit, plus add-ons)</t>
   </si>
   <si>
-    <t xml:space="preserve">early Dec</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RSDS final payment per its terms</t>
+    <t xml:space="preserve">Fri 8 Jan, on site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RSDS balance paid on departure: cash in EUR earns 5% off, card in EGP costs 3% (George carries the club card or a bank draft; decide in December)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">George / club account</t>
   </si>
   <si>
     <t xml:space="preserve">Sun 3 Jan</t>
@@ -487,7 +490,13 @@
     <t xml:space="preserve">Refund ladder</t>
   </si>
   <si>
-    <t xml:space="preserve">Mirror RSDS's cancellation terms once known; until then deposits refundable in full until the club pays RSDS, then only if the place is resold.</t>
+    <t xml:space="preserve">Mirrors RSDS: deposit non-refundable once paid to RSDS (23 Oct); cancellation more than 30 days out costs 20% of the place, 15–29 days 30%, 7–14 days 50%, 6 days or less 80%, no-show 100%; a resold place is refunded in full less the club's costs.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cancellation ladder (RSDS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&gt;30 days 20% / 15–29 days 30% / 7–14 days 50% / &lt;=6 days 80% / no-show 100%; low season 3–8 Jan, no supplements</t>
   </si>
   <si>
     <t xml:space="preserve">Money handling</t>
@@ -1055,7 +1064,7 @@
         <v>26</v>
       </c>
       <c r="B12" s="8" t="n">
-        <v>347</v>
+        <v>308</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>27</v>
@@ -1069,7 +1078,7 @@
         <v>29</v>
       </c>
       <c r="B13" s="8" t="n">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>27</v>
@@ -1162,12 +1171,12 @@
         <v>32</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
         <v>41</v>
       </c>
       <c r="B20" s="8" t="n">
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="C20" s="2" t="s">
         <v>42</v>
@@ -1223,18 +1232,18 @@
         <v>50</v>
       </c>
       <c r="B24" s="7" t="n">
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>15</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B25" s="2"/>
       <c r="C25" s="2"/>
@@ -1242,21 +1251,21 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B26" s="8" t="n">
         <v>1000</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B27" s="8" t="n">
         <f aca="false">Inputs!$B$10*Inputs!$B$11*0.5</f>
@@ -1266,27 +1275,27 @@
         <v>27</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B28" s="8" t="n">
         <f aca="false">Inputs!$B$20*4</f>
-        <v>80</v>
+        <v>156</v>
       </c>
       <c r="C28" s="2" t="s">
         <v>27</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B29" s="2"/>
       <c r="C29" s="2"/>
@@ -1294,7 +1303,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B30" s="8" t="n">
         <v>82</v>
@@ -1303,40 +1312,40 @@
         <v>27</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B31" s="8" t="n">
         <v>84</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B32" s="8" t="n">
         <v>30</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D32" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B33" s="8" t="n">
         <v>45</v>
@@ -1345,7 +1354,7 @@
         <v>27</v>
       </c>
       <c r="D33" s="2" t="s">
-        <v>67</v>
+        <v>30</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1382,7 +1391,7 @@
         <v>50</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>70</v>
@@ -1433,11 +1442,11 @@
       </c>
       <c r="B3" s="9" t="n">
         <f aca="false">Inputs!$B$14+Inputs!$B$15+Inputs!$B$13</f>
-        <v>521</v>
+        <v>529</v>
       </c>
       <c r="C3" s="9" t="n">
         <f aca="false">Inputs!$B$12</f>
-        <v>347</v>
+        <v>308</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1458,11 +1467,11 @@
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">Inputs!$B$20*Inputs!$B$22</f>
-        <v>20</v>
+        <v>39</v>
       </c>
       <c r="C5" s="9" t="n">
         <f aca="false">Inputs!$B$20*Inputs!$B$21</f>
-        <v>80</v>
+        <v>156</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1497,11 +1506,11 @@
       </c>
       <c r="B8" s="9" t="n">
         <f aca="false">(Inputs!$B$26/Inputs!$B$4+Inputs!$B$27+Inputs!$B$28)/(Inputs!$B$5-1)</f>
-        <v>60.3799894415498</v>
+        <v>64.3799894415498</v>
       </c>
       <c r="C8" s="9" t="n">
         <f aca="false">(Inputs!$B$26/Inputs!$B$4+Inputs!$B$27+Inputs!$B$28)/(Inputs!$B$5-1)</f>
-        <v>60.3799894415498</v>
+        <v>64.3799894415498</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1510,11 +1519,11 @@
       </c>
       <c r="B9" s="10" t="n">
         <f aca="false">SUM(B3:B8)</f>
-        <v>1008.37998944155</v>
+        <v>1039.37998944155</v>
       </c>
       <c r="C9" s="10" t="n">
         <f aca="false">SUM(C3:C8)</f>
-        <v>961.37998944155</v>
+        <v>1002.37998944155</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1523,11 +1532,11 @@
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">ROUND(B9*Inputs!$B$8,0)</f>
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">ROUND(C9*Inputs!$B$8,0)</f>
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1536,11 +1545,11 @@
       </c>
       <c r="B11" s="9" t="n">
         <f aca="false">(B9+B10)*Inputs!$B$4</f>
-        <v>1226.04415789474</v>
+        <v>1262.73215789474</v>
       </c>
       <c r="C11" s="9" t="n">
         <f aca="false">(C9+C10)*Inputs!$B$4</f>
-        <v>1168.71915789474</v>
+        <v>1218.01865789474</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1548,12 +1557,12 @@
         <v>86</v>
       </c>
       <c r="B12" s="10" t="n">
-        <f aca="false">CEILING(B11,100)</f>
+        <f aca="false">CEILING(B11,50)</f>
         <v>1300</v>
       </c>
       <c r="C12" s="10" t="n">
-        <f aca="false">CEILING(C11,100)</f>
-        <v>1200</v>
+        <f aca="false">CEILING(C11,50)</f>
+        <v>1250</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1627,7 +1636,7 @@
       </c>
       <c r="C20" s="10" t="n">
         <f aca="false">C12</f>
-        <v>1200</v>
+        <v>1250</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1653,7 +1662,7 @@
       </c>
       <c r="C22" s="10" t="n">
         <f aca="false">C20+C21</f>
-        <v>1609.6055</v>
+        <v>1659.6055</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1665,7 +1674,7 @@
       </c>
       <c r="C23" s="10" t="n">
         <f aca="false">C22+C15+C16</f>
-        <v>1978.7785</v>
+        <v>2028.7785</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1843,19 +1852,19 @@
       </c>
       <c r="B9" s="10" t="n">
         <f aca="false">(B5*Fee!$B$12+B6*Fee!$C$12)/Inputs!$B$4</f>
-        <v>12036.6332315744</v>
+        <v>12254.6881814217</v>
       </c>
       <c r="C9" s="10" t="n">
         <f aca="false">(C5*Fee!$B$12+C6*Fee!$C$12)/Inputs!$B$4</f>
-        <v>20758.8312254688</v>
+        <v>21151.3301351941</v>
       </c>
       <c r="D9" s="10" t="n">
         <f aca="false">(D5*Fee!$B$12+D6*Fee!$C$12)/Inputs!$B$4</f>
-        <v>26166.5939816834</v>
+        <v>26689.9258613171</v>
       </c>
       <c r="E9" s="10" t="n">
         <f aca="false">(E5*Fee!$B$12+E6*Fee!$C$12)/Inputs!$B$4</f>
-        <v>31661.5787178369</v>
+        <v>32272.1325774095</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1894,19 +1903,19 @@
       </c>
       <c r="B12" s="9" t="n">
         <f aca="false">B5*(Inputs!$B$14+Inputs!$B$15+Inputs!$B$13)</f>
-        <v>3126</v>
+        <v>3174</v>
       </c>
       <c r="C12" s="9" t="n">
         <f aca="false">C5*(Inputs!$B$14+Inputs!$B$15+Inputs!$B$13)</f>
-        <v>5210</v>
+        <v>5290</v>
       </c>
       <c r="D12" s="9" t="n">
         <f aca="false">D5*(Inputs!$B$14+Inputs!$B$15+Inputs!$B$13)</f>
-        <v>6252</v>
+        <v>6348</v>
       </c>
       <c r="E12" s="9" t="n">
         <f aca="false">E5*(Inputs!$B$14+Inputs!$B$15+Inputs!$B$13)</f>
-        <v>7815</v>
+        <v>7935</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1915,19 +1924,19 @@
       </c>
       <c r="B13" s="9" t="n">
         <f aca="false">B6*(Inputs!$B$12+Inputs!$B$17)</f>
-        <v>2070</v>
+        <v>1875</v>
       </c>
       <c r="C13" s="9" t="n">
         <f aca="false">C6*(Inputs!$B$12+Inputs!$B$17)</f>
-        <v>3726</v>
+        <v>3375</v>
       </c>
       <c r="D13" s="9" t="n">
         <f aca="false">D6*(Inputs!$B$12+Inputs!$B$17)</f>
-        <v>4968</v>
+        <v>4500</v>
       </c>
       <c r="E13" s="9" t="n">
         <f aca="false">E6*(Inputs!$B$12+Inputs!$B$17)</f>
-        <v>5796</v>
+        <v>5250</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1965,11 +1974,11 @@
       </c>
       <c r="D15" s="9" t="n">
         <f aca="false">-MAX(D7-1,0)*(Inputs!$B$10*Inputs!$B$11+Inputs!$B$12)</f>
-        <v>-737</v>
+        <v>-698</v>
       </c>
       <c r="E15" s="9" t="n">
         <f aca="false">-MAX(E7-1,0)*(Inputs!$B$10*Inputs!$B$11+Inputs!$B$12)</f>
-        <v>-737</v>
+        <v>-698</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1999,19 +2008,19 @@
       </c>
       <c r="B17" s="10" t="n">
         <f aca="false">B11+B12+B13+B14+B15+B16</f>
-        <v>9690</v>
+        <v>9543</v>
       </c>
       <c r="C17" s="10" t="n">
         <f aca="false">C11+C12+C13+C14+C15+C16</f>
-        <v>16686</v>
+        <v>16415</v>
       </c>
       <c r="D17" s="10" t="n">
         <f aca="false">D11+D12+D13+D14+D15+D16</f>
-        <v>20268</v>
+        <v>19935</v>
       </c>
       <c r="E17" s="10" t="n">
         <f aca="false">E11+E12+E13+E14+E15+E16</f>
-        <v>24694</v>
+        <v>24307</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2020,19 +2029,19 @@
       </c>
       <c r="B18" s="9" t="n">
         <f aca="false">(B6+1)*Inputs!$B$20*Inputs!$B$21+B5*Inputs!$B$20*Inputs!$B$22</f>
-        <v>600</v>
+        <v>1170</v>
       </c>
       <c r="C18" s="9" t="n">
         <f aca="false">(C6+1)*Inputs!$B$20*Inputs!$B$21+C5*Inputs!$B$20*Inputs!$B$22</f>
-        <v>1000</v>
+        <v>1950</v>
       </c>
       <c r="D18" s="9" t="n">
         <f aca="false">(D6+1)*Inputs!$B$20*Inputs!$B$21+D5*Inputs!$B$20*Inputs!$B$22</f>
-        <v>1280</v>
+        <v>2496</v>
       </c>
       <c r="E18" s="9" t="n">
         <f aca="false">(E6+1)*Inputs!$B$20*Inputs!$B$21+E5*Inputs!$B$20*Inputs!$B$22</f>
-        <v>1500</v>
+        <v>2925</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2083,19 +2092,19 @@
       </c>
       <c r="B21" s="10" t="n">
         <f aca="false">B17+B18+B19+B20</f>
-        <v>11162.2197993894</v>
+        <v>11585.2197993894</v>
       </c>
       <c r="C21" s="10" t="n">
         <f aca="false">C17+C18+C19+C20</f>
-        <v>18558.2197993894</v>
+        <v>19237.2197993894</v>
       </c>
       <c r="D21" s="10" t="n">
         <f aca="false">D17+D18+D19+D20</f>
-        <v>22615.2197993894</v>
+        <v>23498.2197993894</v>
       </c>
       <c r="E21" s="10" t="n">
         <f aca="false">E17+E18+E19+E20</f>
-        <v>27066.2197993894</v>
+        <v>28104.2197993894</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2113,19 +2122,19 @@
       </c>
       <c r="B23" s="10" t="n">
         <f aca="false">B9-B21</f>
-        <v>874.413432184911</v>
+        <v>669.468382032272</v>
       </c>
       <c r="C23" s="10" t="n">
         <f aca="false">C9-C21</f>
-        <v>2200.61142607937</v>
+        <v>1914.11033580462</v>
       </c>
       <c r="D23" s="10" t="n">
         <f aca="false">D9-D21</f>
-        <v>3551.37418229394</v>
+        <v>3191.70606192761</v>
       </c>
       <c r="E23" s="10" t="n">
         <f aca="false">E9-E21</f>
-        <v>4595.35891844745</v>
+        <v>4167.91277802006</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2134,19 +2143,19 @@
       </c>
       <c r="B24" s="9" t="n">
         <f aca="false">B23*Inputs!$B$4</f>
-        <v>1002.515</v>
+        <v>767.5455</v>
       </c>
       <c r="C24" s="9" t="n">
         <f aca="false">C23*Inputs!$B$4</f>
-        <v>2523.001</v>
+        <v>2194.5275</v>
       </c>
       <c r="D24" s="9" t="n">
         <f aca="false">D23*Inputs!$B$4</f>
-        <v>4071.6505</v>
+        <v>3659.291</v>
       </c>
       <c r="E24" s="9" t="n">
         <f aca="false">E23*Inputs!$B$4</f>
-        <v>5268.579</v>
+        <v>4778.512</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2184,14 +2193,14 @@
       </c>
       <c r="D26" s="10" t="n">
         <f aca="false">-D15</f>
-        <v>737</v>
+        <v>698</v>
       </c>
       <c r="E26" s="10" t="n">
         <f aca="false">-E15</f>
-        <v>737</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
         <v>127</v>
       </c>
@@ -2227,19 +2236,19 @@
       </c>
       <c r="B29" s="9" t="n">
         <f aca="false">B17*Inputs!$B$24</f>
-        <v>2422.5</v>
+        <v>1908.6</v>
       </c>
       <c r="C29" s="9" t="n">
         <f aca="false">C17*Inputs!$B$24</f>
-        <v>4171.5</v>
+        <v>3283</v>
       </c>
       <c r="D29" s="9" t="n">
         <f aca="false">D17*Inputs!$B$24</f>
-        <v>5067</v>
+        <v>3987</v>
       </c>
       <c r="E29" s="9" t="n">
         <f aca="false">E17*Inputs!$B$24</f>
-        <v>6173.5</v>
+        <v>4861.4</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2248,22 +2257,22 @@
       </c>
       <c r="B30" s="10" t="n">
         <f aca="false">B28-B29</f>
-        <v>1415.26711731356</v>
+        <v>1929.16711731356</v>
       </c>
       <c r="C30" s="10" t="n">
         <f aca="false">C28-C29</f>
-        <v>2457.37047535979</v>
+        <v>3345.87047535979</v>
       </c>
       <c r="D30" s="10" t="n">
         <f aca="false">D28-D29</f>
-        <v>3306.31007413868</v>
+        <v>4386.31007413868</v>
       </c>
       <c r="E30" s="10" t="n">
         <f aca="false">E28-E29</f>
-        <v>3944.24967291757</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>5256.34967291757</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="2" t="s">
         <v>131</v>
       </c>
@@ -2288,7 +2297,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22"/>
@@ -2296,7 +2305,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="24"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="76.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="61.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>132</v>
       </c>
@@ -2336,7 +2345,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="2" t="s">
         <v>142</v>
       </c>
@@ -2358,7 +2367,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="s">
         <v>147</v>
       </c>
@@ -2366,15 +2375,15 @@
         <v>148</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="2" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>141</v>
@@ -2382,10 +2391,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="2" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>144</v>
@@ -2396,25 +2405,36 @@
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
     </row>
-    <row r="11" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="2" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C12" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="2" t="s">
+        <v>158</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>159</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>